<commit_message>
fixed handling of indefinite LED "ON"; closes #4
</commit_message>
<xml_diff>
--- a/diagrams/juryFull/BlueOwl-Jury.xlsx
+++ b/diagrams/juryFull/BlueOwl-Jury.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\owlcms\devices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E167CBF-3CF7-4ADB-AC9C-672E0709E873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BA2F03-13EA-48FB-A45D-772B844DCC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F9C8F068-60C0-4FDD-8C1E-880F519290ED}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F9C8F068-60C0-4FDD-8C1E-880F519290ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Jury" sheetId="2" r:id="rId1"/>
@@ -1673,7 +1673,7 @@
         <v>169</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>3</v>
@@ -1690,7 +1690,7 @@
         <v>169</v>
       </c>
       <c r="D42" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>4</v>
@@ -1707,7 +1707,7 @@
         <v>169</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>4</v>
@@ -1724,7 +1724,7 @@
         <v>169</v>
       </c>
       <c r="D44" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>3</v>
@@ -1741,7 +1741,7 @@
         <v>169</v>
       </c>
       <c r="D45" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>3</v>
@@ -1758,7 +1758,7 @@
         <v>169</v>
       </c>
       <c r="D46" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>3</v>
@@ -2912,7 +2912,7 @@
         <v>95</v>
       </c>
       <c r="B118" s="10">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C118" t="s">
         <v>168</v>
@@ -2965,7 +2965,7 @@
         <v>110</v>
       </c>
       <c r="B121" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>170</v>
@@ -3016,7 +3016,7 @@
         <v>125</v>
       </c>
       <c r="B124" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>170</v>
@@ -3067,7 +3067,7 @@
         <v>140</v>
       </c>
       <c r="B127" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>170</v>
@@ -3115,7 +3115,7 @@
         <v>155</v>
       </c>
       <c r="B130" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>167</v>
@@ -3157,7 +3157,7 @@
         <v>155</v>
       </c>
       <c r="B133" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C133" t="s">
         <v>171</v>
@@ -3199,7 +3199,7 @@
         <v>155</v>
       </c>
       <c r="B136" s="9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C136" t="s">
         <v>172</v>

</xml_diff>